<commit_message>
Stop template placeholders from leaking into exported summaries
The xlsx templates carried example values in every data cell of row 10
(company name "Альфа", insurance sum 2 000 000, premium 100 000 / 75 000,
franchise 50 000, etc.). The export writes cells conditionally, so any
branch that skipped a write (missing premium, failed validation, no
second variant in another offer of a mixed summary) left the example
values visible in the downloaded file.

Two-layer defence:
- Strip the example values from all four summary templates, keeping the
  cell formulas (rate, premium sums) and formatting intact.
- Add ExcelExportService._clear_row_data_values, invoked from
  _fill_company_data_row after style copy and before any write, which
  blanks every mapped data cell that is not a formula. Future templates
  with placeholders, or new conditional branches, can no longer leak.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/client_summary_template.xlsx
+++ b/templates/client_summary_template.xlsx
@@ -1,261 +1,172 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grachev\Yandex.Disk\Работа\ОнлайнБрокер\soft\onlineservice\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82F8895-EADA-46A4-ADF7-909CC432F704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="summary_template_sheet" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary_template_sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">summary_template_sheet!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'summary_template_sheet'!$A$1:$Q$11</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
-  <si>
-    <t>Свод котировок и условий по заявке №</t>
-  </si>
-  <si>
-    <t>23459-ЛА-КЗ</t>
-  </si>
-  <si>
-    <t>Объект страхования</t>
-  </si>
-  <si>
-    <t>Haval Jolion</t>
-  </si>
-  <si>
-    <t>Лизингополучатель</t>
-  </si>
-  <si>
-    <t>ООО "Ромашка"</t>
-  </si>
-  <si>
-    <t>Предложение 1</t>
-  </si>
-  <si>
-    <t>ИТОГО</t>
-  </si>
-  <si>
-    <t>Предложение 2</t>
-  </si>
-  <si>
-    <t>Страховая компания</t>
-  </si>
-  <si>
-    <t>срок</t>
-  </si>
-  <si>
-    <t>СС</t>
-  </si>
-  <si>
-    <t>тариф</t>
-  </si>
-  <si>
-    <t>CП</t>
-  </si>
-  <si>
-    <t>франшиза</t>
-  </si>
-  <si>
-    <t>Комментарии</t>
-  </si>
-  <si>
-    <t>Альфа</t>
-  </si>
-  <si>
-    <t>1 год</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Выбрана СК:</t>
-  </si>
-  <si>
-    <t>Выбрано предложение:</t>
-  </si>
-  <si>
-    <t>Цели использования</t>
-  </si>
-  <si>
-    <t>Сравнительный анализ страховых тарифов</t>
-  </si>
-  <si>
-    <t>Примечание:</t>
-  </si>
-  <si>
-    <t>платежей в год</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="19">
     <font>
+      <name val="Arial Cyr"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial Cyr"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="8"/>
       <sz val="14"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="8"/>
       <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="14"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="13"/>
       <sz val="11"/>
-      <color indexed="13"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="12"/>
       <sz val="14"/>
-      <color indexed="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="13"/>
       <sz val="12"/>
-      <color indexed="13"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="12"/>
       <sz val="11"/>
-      <color indexed="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="20"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="16"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="8"/>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <i/>
+      <name val="Arial"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
-      <i/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color indexed="8"/>
       <sz val="14"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <i/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color indexed="8"/>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
     <font>
-      <i/>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="14">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -430,180 +341,182 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5"/>
   </cellStyleXfs>
-  <cellXfs count="63">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="66">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="8" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="8" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="12" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="12" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="12" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="12" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="12" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="14" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="12" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -672,14 +585,6 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -1757,390 +1662,403 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="34.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="2.85546875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13" style="3" customWidth="1"/>
-    <col min="10" max="10" width="2.85546875" style="3" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="3" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" style="3" customWidth="1"/>
-    <col min="14" max="14" width="15" style="3" customWidth="1"/>
-    <col min="15" max="15" width="13" style="3" customWidth="1"/>
-    <col min="16" max="16" width="2.85546875" style="3" customWidth="1"/>
-    <col min="17" max="17" width="29.5703125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="2.85546875" style="3" customWidth="1"/>
-    <col min="19" max="20" width="13.5703125" style="3" customWidth="1"/>
-    <col min="21" max="21" width="9" style="3" customWidth="1"/>
-    <col min="22" max="16384" width="9" style="3"/>
+    <col width="34.42578125" customWidth="1" style="3" min="1" max="1"/>
+    <col width="15.42578125" customWidth="1" style="3" min="2" max="2"/>
+    <col width="22.85546875" customWidth="1" style="3" min="3" max="3"/>
+    <col width="2.85546875" customWidth="1" style="3" min="4" max="4"/>
+    <col width="11.85546875" customWidth="1" style="3" min="5" max="5"/>
+    <col width="13.5703125" customWidth="1" style="3" min="6" max="6"/>
+    <col width="14.7109375" customWidth="1" style="3" min="7" max="7"/>
+    <col width="14.28515625" customWidth="1" style="3" min="8" max="8"/>
+    <col width="13" customWidth="1" style="3" min="9" max="9"/>
+    <col width="2.85546875" customWidth="1" style="3" min="10" max="10"/>
+    <col width="13.5703125" customWidth="1" style="3" min="11" max="11"/>
+    <col width="14.85546875" customWidth="1" style="3" min="12" max="12"/>
+    <col width="14.7109375" customWidth="1" style="3" min="13" max="13"/>
+    <col width="15" customWidth="1" style="3" min="14" max="14"/>
+    <col width="13" customWidth="1" style="3" min="15" max="15"/>
+    <col width="2.85546875" customWidth="1" style="3" min="16" max="16"/>
+    <col width="29.5703125" customWidth="1" style="3" min="17" max="17"/>
+    <col width="2.85546875" customWidth="1" style="3" min="18" max="18"/>
+    <col width="13.5703125" customWidth="1" style="3" min="19" max="20"/>
+    <col width="9" customWidth="1" style="3" min="21" max="21"/>
+    <col width="9" customWidth="1" style="3" min="22" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="57" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="R1" s="2"/>
-      <c r="S1" s="59"/>
-      <c r="T1" s="61"/>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>Свод котировок и условий по заявке №</t>
+        </is>
+      </c>
+      <c r="B1" s="63" t="n"/>
+      <c r="C1" s="57" t="inlineStr">
+        <is>
+          <t>23459-ЛА-КЗ</t>
+        </is>
+      </c>
+      <c r="D1" s="63" t="n"/>
+      <c r="E1" s="63" t="n"/>
+      <c r="F1" s="63" t="n"/>
+      <c r="G1" s="63" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="59" t="n"/>
+      <c r="L1" s="63" t="n"/>
+      <c r="M1" s="63" t="n"/>
+      <c r="N1" s="63" t="n"/>
+      <c r="O1" s="59" t="n"/>
+      <c r="P1" s="59" t="n"/>
+      <c r="Q1" s="41" t="inlineStr">
+        <is>
+          <t>Выбрана СК:</t>
+        </is>
+      </c>
+      <c r="R1" s="59" t="n"/>
+      <c r="S1" s="61" t="n"/>
+      <c r="T1" s="64" t="n"/>
     </row>
-    <row r="2" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="49" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="60"/>
-      <c r="T2" s="62"/>
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>Объект страхования</t>
+        </is>
+      </c>
+      <c r="C2" s="49" t="inlineStr">
+        <is>
+          <t>Haval Jolion</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
+      <c r="O2" s="60" t="n"/>
+      <c r="P2" s="60" t="n"/>
+      <c r="Q2" s="36" t="n"/>
+      <c r="R2" s="60" t="n"/>
+      <c r="T2" s="65" t="n"/>
     </row>
-    <row r="3" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="47" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="6"/>
+    <row r="3" ht="18.75" customHeight="1">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Лизингополучатель</t>
+        </is>
+      </c>
+      <c r="C3" s="49" t="inlineStr">
+        <is>
+          <t>ООО "Ромашка"</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="42" t="inlineStr">
+        <is>
+          <t>Выбрано предложение:</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
+      <c r="T3" s="6" t="n"/>
     </row>
-    <row r="4" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="51" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="37"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="6"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Цели использования</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="37" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
+      <c r="T4" s="6" t="n"/>
     </row>
-    <row r="5" spans="1:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="43" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="40"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="38"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="6"/>
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Примечание:</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="n"/>
+      <c r="E5" s="39" t="n"/>
+      <c r="F5" s="39" t="n"/>
+      <c r="G5" s="39" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="38" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="6" t="n"/>
     </row>
-    <row r="6" spans="1:20" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="9"/>
+    <row r="6" ht="8.25" customHeight="1">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="8" t="n"/>
+      <c r="N6" s="8" t="n"/>
+      <c r="O6" s="8" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="9" t="n"/>
     </row>
-    <row r="7" spans="1:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="10"/>
-      <c r="K7" s="45" t="s">
-        <v>8</v>
-      </c>
-      <c r="L7" s="46"/>
-      <c r="M7" s="46"/>
-      <c r="N7" s="46"/>
-      <c r="O7" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="9"/>
+    <row r="7" ht="31.5" customHeight="1">
+      <c r="A7" s="53" t="inlineStr">
+        <is>
+          <t>Сравнительный анализ страховых тарифов</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>Предложение 1</t>
+        </is>
+      </c>
+      <c r="I7" s="45" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="45" t="inlineStr">
+        <is>
+          <t>Предложение 2</t>
+        </is>
+      </c>
+      <c r="O7" s="45" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="n"/>
+      <c r="Q7" s="10" t="n"/>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="9" t="n"/>
     </row>
-    <row r="8" spans="1:20" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I8" s="46"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="M8" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="O8" s="46"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="R8" s="13"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="15"/>
+    <row r="8" ht="41.25" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Страховая компания</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>срок</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>СС</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>тариф</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>CП</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>франшиза</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>платежей в год</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="n"/>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>тариф</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>CП</t>
+        </is>
+      </c>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>франшиза</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
+          <t>платежей в год</t>
+        </is>
+      </c>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="14" t="inlineStr">
+        <is>
+          <t>Комментарии</t>
+        </is>
+      </c>
+      <c r="R8" s="13" t="n"/>
+      <c r="S8" s="4" t="n"/>
+      <c r="T8" s="15" t="n"/>
     </row>
-    <row r="9" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="20"/>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="16" t="n"/>
+      <c r="B9" s="17" t="n"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="17" t="n"/>
+      <c r="L9" s="17" t="n"/>
+      <c r="M9" s="17" t="n"/>
+      <c r="N9" s="17" t="n"/>
+      <c r="O9" s="17" t="n"/>
+      <c r="P9" s="18" t="n"/>
+      <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="18" t="n"/>
+      <c r="S9" s="4" t="n"/>
+      <c r="T9" s="20" t="n"/>
     </row>
-    <row r="10" spans="1:20" ht="26.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="35">
-        <v>2000000</v>
-      </c>
-      <c r="D10" s="18"/>
+    <row r="10" ht="26.25" customHeight="1">
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="34" t="n"/>
+      <c r="C10" s="35" t="n"/>
+      <c r="D10" s="18" t="n"/>
       <c r="E10" s="27">
         <f>F10/C10</f>
-        <v>0.05</v>
-      </c>
-      <c r="F10" s="28">
-        <v>100000</v>
-      </c>
-      <c r="G10" s="29">
-        <v>0</v>
-      </c>
-      <c r="H10" s="29">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F10" s="28" t="n"/>
+      <c r="G10" s="29" t="n"/>
+      <c r="H10" s="29" t="n"/>
       <c r="I10" s="22">
         <f>SUM(F10:F10)</f>
-        <v>100000</v>
-      </c>
-      <c r="J10" s="18"/>
+        <v/>
+      </c>
+      <c r="J10" s="18" t="n"/>
       <c r="K10" s="30">
         <f>L10/C10</f>
-        <v>3.7499999999999999E-2</v>
-      </c>
-      <c r="L10" s="31">
-        <v>75000</v>
-      </c>
-      <c r="M10" s="32">
-        <v>50000</v>
-      </c>
-      <c r="N10" s="33">
-        <v>1</v>
-      </c>
+        <v/>
+      </c>
+      <c r="L10" s="31" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="33" t="n"/>
       <c r="O10" s="22">
         <f>SUM(L10:L10)</f>
-        <v>75000</v>
-      </c>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="R10" s="18"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="20"/>
+        <v/>
+      </c>
+      <c r="P10" s="18" t="n"/>
+      <c r="Q10" s="23" t="n"/>
+      <c r="R10" s="18" t="n"/>
+      <c r="S10" s="4" t="n"/>
+      <c r="T10" s="20" t="n"/>
     </row>
-    <row r="11" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="26"/>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="24" t="n"/>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="25" t="n"/>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="25" t="n"/>
+      <c r="G11" s="25" t="n"/>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="25" t="n"/>
+      <c r="L11" s="25" t="n"/>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="25" t="n"/>
+      <c r="O11" s="25" t="n"/>
+      <c r="P11" s="25" t="n"/>
+      <c r="Q11" s="25" t="n"/>
+      <c r="R11" s="25" t="n"/>
+      <c r="S11" s="25" t="n"/>
+      <c r="T11" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="S1:T2"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="K7:N7"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="I7:I8"/>
     <mergeCell ref="K1:N2"/>
-    <mergeCell ref="S1:T2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="K7:N7"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="50" orientation="landscape" r:id="rId1"/>
+  <pageSetup orientation="landscape" scale="50"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial Cyr,Regular"&amp;10&amp;K000000summary_template.xlsx&amp;C&amp;"Helvetica Neue,Regular"&amp;11&amp;K000000&amp;P</oddHeader>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;11&amp;K000000&amp;P</oddFooter>
+    <oddHeader>&amp;L&amp;"Arial Cyr,Regular"&amp;10 &amp;K000000summary_template.xlsx&amp;C&amp;"Helvetica Neue,Regular"&amp;11 &amp;K000000&amp;P</oddHeader>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;11 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>